<commit_message>
Ajustar presupuesto: imprevistos 5% solo sobre materiales y lamina del porton a 1 mm
- Imprevistos (5%) se calculan unicamente sobre el subtotal de materiales,
  no sobre materiales + mano de obra.
- Lamina negra del porton corregida a 1 mm (cal. 20) segun la lista; precio
  ajustado a C$ 1,250. Especificacion tecnica actualizada.
- Nuevo total general: C$ 53,706.35.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018cUG4L4bYGYeGqZHWF8NkF
</commit_message>
<xml_diff>
--- a/Presupuesto_Muro_Perimetral.xlsx
+++ b/Presupuesto_Muro_Perimetral.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Presupuesto'!$11:$11</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Presupuesto'!$A$1:$F$68</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Presupuesto'!$A$1:$F$67</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Especificaciones Técnicas'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Especificaciones Técnicas'!$A$1:$D$21</definedName>
   </definedNames>
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>Lámina negra de 4x8 pies x 1/16"</t>
+          <t>Lámina negra de 4x8 pies x 1 mm (cal. 20)</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
@@ -1337,11 +1337,11 @@
         <v>1</v>
       </c>
       <c r="E33" s="12" t="n">
-        <v>1600</v>
+        <v>1250</v>
       </c>
       <c r="F33" s="13">
         <f>D33*E33</f>
-        <v>1600</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="34" ht="21" customHeight="1">
@@ -1431,7 +1431,7 @@
       <c r="E37" s="15" t="n"/>
       <c r="F37" s="16">
         <f>SUM(F27:F36)</f>
-        <v>12280</v>
+        <v>11930</v>
       </c>
     </row>
     <row r="38" ht="24" customHeight="1">
@@ -1567,13 +1567,13 @@
       <c r="E45" s="15" t="n"/>
       <c r="F45" s="24">
         <f>F24+F37</f>
-        <v>36737</v>
+        <v>36387</v>
       </c>
     </row>
     <row r="46" ht="22" customHeight="1">
       <c r="A46" s="23" t="inlineStr">
         <is>
-          <t>Subtotal mano de obra</t>
+          <t>Imprevistos (5% sobre materiales)</t>
         </is>
       </c>
       <c r="B46" s="15" t="n"/>
@@ -1581,93 +1581,90 @@
       <c r="D46" s="15" t="n"/>
       <c r="E46" s="15" t="n"/>
       <c r="F46" s="24">
-        <f>F42</f>
-        <v>15500</v>
+        <f>F45*0.05</f>
+        <v>1819.35</v>
       </c>
     </row>
     <row r="47" ht="22" customHeight="1">
-      <c r="A47" s="14" t="inlineStr">
-        <is>
-          <t>Subtotal general</t>
+      <c r="A47" s="23" t="inlineStr">
+        <is>
+          <t>Subtotal mano de obra</t>
         </is>
       </c>
       <c r="B47" s="15" t="n"/>
       <c r="C47" s="15" t="n"/>
       <c r="D47" s="15" t="n"/>
       <c r="E47" s="15" t="n"/>
-      <c r="F47" s="16">
-        <f>F45+F46</f>
-        <v>52237</v>
-      </c>
-    </row>
-    <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="14" t="inlineStr">
-        <is>
-          <t>Imprevistos (5%)</t>
-        </is>
-      </c>
-      <c r="B48" s="15" t="n"/>
-      <c r="C48" s="15" t="n"/>
-      <c r="D48" s="15" t="n"/>
-      <c r="E48" s="15" t="n"/>
-      <c r="F48" s="16">
-        <f>F47*0.05</f>
-        <v>2611.85</v>
-      </c>
-    </row>
-    <row r="49" ht="26" customHeight="1">
-      <c r="A49" s="25" t="inlineStr">
+      <c r="F47" s="24">
+        <f>F42</f>
+        <v>15500</v>
+      </c>
+    </row>
+    <row r="48" ht="26" customHeight="1">
+      <c r="A48" s="25" t="inlineStr">
         <is>
           <t>TOTAL GENERAL (C$)</t>
         </is>
       </c>
-      <c r="B49" s="26" t="n"/>
-      <c r="C49" s="26" t="n"/>
-      <c r="D49" s="26" t="n"/>
-      <c r="E49" s="26" t="n"/>
-      <c r="F49" s="27">
-        <f>F47+F48</f>
-        <v>54848.85</v>
+      <c r="B48" s="26" t="n"/>
+      <c r="C48" s="26" t="n"/>
+      <c r="D48" s="26" t="n"/>
+      <c r="E48" s="26" t="n"/>
+      <c r="F48" s="27">
+        <f>F45+F46+F47</f>
+        <v>53706.35</v>
+      </c>
+    </row>
+    <row r="49" ht="16" customHeight="1">
+      <c r="A49" s="28" t="inlineStr">
+        <is>
+          <t>IVA (15%) ya contenido en el monto de materiales:</t>
+        </is>
+      </c>
+      <c r="F49" s="29">
+        <f>(F24+F37)/1.15*0.15</f>
+        <v>4746.13</v>
       </c>
     </row>
     <row r="50" ht="16" customHeight="1">
       <c r="A50" s="28" t="inlineStr">
         <is>
-          <t>IVA (15%) ya contenido en el monto de materiales:</t>
-        </is>
-      </c>
-      <c r="F50" s="29">
-        <f>(F24+F37)/1.15*0.15</f>
-        <v>4791.78</v>
-      </c>
-    </row>
-    <row r="51" ht="16" customHeight="1">
-      <c r="A51" s="28" t="inlineStr">
-        <is>
           <t>Total general equivalente en dólares (referencial, no vinculante):</t>
         </is>
       </c>
-      <c r="F51" s="30">
-        <f>F49/36.62</f>
-        <v>1497.78</v>
-      </c>
-    </row>
-    <row r="53" ht="24" customHeight="1">
-      <c r="A53" s="21" t="inlineStr">
+      <c r="F50" s="30">
+        <f>F48/36.62</f>
+        <v>1466.59</v>
+      </c>
+    </row>
+    <row r="52" ht="24" customHeight="1">
+      <c r="A52" s="21" t="inlineStr">
         <is>
           <t>OBSERVACIONES</t>
         </is>
       </c>
-      <c r="B53" s="22" t="n"/>
-      <c r="C53" s="22" t="n"/>
-      <c r="D53" s="22" t="n"/>
-      <c r="E53" s="22" t="n"/>
-      <c r="F53" s="22" t="n"/>
+      <c r="B52" s="22" t="n"/>
+      <c r="C52" s="22" t="n"/>
+      <c r="D52" s="22" t="n"/>
+      <c r="E52" s="22" t="n"/>
+      <c r="F52" s="22" t="n"/>
+    </row>
+    <row r="53" ht="36" customHeight="1">
+      <c r="A53" s="31" t="inlineStr">
+        <is>
+          <t>1. Precios unitarios según el mercado de ferreterías de Managua, Nicaragua (agosto 2026); incluyen IVA (15%). Están sujetos a variación por disponibilidad y fluctuación del mercado.</t>
+        </is>
+      </c>
+      <c r="B53" s="32" t="n"/>
+      <c r="C53" s="32" t="n"/>
+      <c r="D53" s="32" t="n"/>
+      <c r="E53" s="32" t="n"/>
+      <c r="F53" s="32" t="n"/>
     </row>
     <row r="54" ht="36" customHeight="1">
       <c r="A54" s="31" t="inlineStr">
         <is>
-          <t>1. Precios unitarios según el mercado de ferreterías de Managua, Nicaragua (agosto 2026); incluyen IVA (15%). Están sujetos a variación por disponibilidad y fluctuación del mercado.</t>
+          <t>2. El muro se levanta sobre un muro de cantera existente y se continúa con bloque de 6" en mampostería confinada (columnas y viga corona de amarre con refuerzo de 3/8" y estribos de 1/4").</t>
         </is>
       </c>
       <c r="B54" s="32" t="n"/>
@@ -1679,7 +1676,7 @@
     <row r="55" ht="36" customHeight="1">
       <c r="A55" s="31" t="inlineStr">
         <is>
-          <t>2. El muro se levanta sobre un muro de cantera existente y se continúa con bloque de 6" en mampostería confinada (columnas y viga corona de amarre con refuerzo de 3/8" y estribos de 1/4").</t>
+          <t>3. Las cantidades provienen de la lista entregada por el cliente. No se incluye desperdicio adicional al 5% de imprevistos ni acarreo de materiales fuera del sitio.</t>
         </is>
       </c>
       <c r="B55" s="32" t="n"/>
@@ -1691,7 +1688,7 @@
     <row r="56" ht="36" customHeight="1">
       <c r="A56" s="31" t="inlineStr">
         <is>
-          <t>3. Las cantidades provienen de la lista entregada por el cliente. No se incluye desperdicio adicional al 5% de imprevistos ni acarreo de materiales fuera del sitio.</t>
+          <t>4. No incluye: excavación o refuerzo de cimiento nuevo, trazo topográfico, permisos municipales, ni acabado fino (repello/afinado), salvo indicación contraria.</t>
         </is>
       </c>
       <c r="B56" s="32" t="n"/>
@@ -1703,7 +1700,7 @@
     <row r="57" ht="36" customHeight="1">
       <c r="A57" s="31" t="inlineStr">
         <is>
-          <t>4. No incluye: excavación o refuerzo de cimiento nuevo, trazo topográfico, permisos municipales, ni acabado fino (repello/afinado), salvo indicación contraria.</t>
+          <t>5. La mano de obra es por trato (precio global) con maestro de obra; no incluye prestaciones de ley ni alimentación, salvo acuerdo por escrito.</t>
         </is>
       </c>
       <c r="B57" s="32" t="n"/>
@@ -1715,7 +1712,7 @@
     <row r="58" ht="36" customHeight="1">
       <c r="A58" s="31" t="inlineStr">
         <is>
-          <t>5. La mano de obra es por trato (precio global) con maestro de obra; no incluye prestaciones de ley ni alimentación, salvo acuerdo por escrito.</t>
+          <t>6. La madera (tablas y reglas) es para formaleta/encofrado de columnas y viga; es material reutilizable no consumido en su totalidad.</t>
         </is>
       </c>
       <c r="B58" s="32" t="n"/>
@@ -1727,7 +1724,7 @@
     <row r="59" ht="36" customHeight="1">
       <c r="A59" s="31" t="inlineStr">
         <is>
-          <t>6. La madera (tablas y reglas) es para formaleta/encofrado de columnas y viga; es material reutilizable no consumido en su totalidad.</t>
+          <t>7. Validez de la oferta: 30 días calendario a partir de la fecha de emisión. Tipo de cambio referencial: 1 USD ≈ C$ 36.62.</t>
         </is>
       </c>
       <c r="B59" s="32" t="n"/>
@@ -1736,34 +1733,38 @@
       <c r="E59" s="32" t="n"/>
       <c r="F59" s="32" t="n"/>
     </row>
-    <row r="60" ht="36" customHeight="1">
-      <c r="A60" s="31" t="inlineStr">
-        <is>
-          <t>7. Validez de la oferta: 30 días calendario a partir de la fecha de emisión. Tipo de cambio referencial: 1 USD ≈ C$ 36.62.</t>
-        </is>
-      </c>
-      <c r="B60" s="32" t="n"/>
-      <c r="C60" s="32" t="n"/>
-      <c r="D60" s="32" t="n"/>
-      <c r="E60" s="32" t="n"/>
-      <c r="F60" s="32" t="n"/>
-    </row>
-    <row r="62" ht="20" customHeight="1">
-      <c r="A62" s="33" t="inlineStr">
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="33" t="inlineStr">
         <is>
           <t>LEYENDA DE COLORES</t>
         </is>
       </c>
     </row>
+    <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="34" t="inlineStr">
+        <is>
+          <t>Texto azul</t>
+        </is>
+      </c>
+      <c r="B62" s="35" t="inlineStr">
+        <is>
+          <t>Celdas editables por el usuario (cantidad y precio unitario). El total se calcula automáticamente.</t>
+        </is>
+      </c>
+      <c r="C62" s="32" t="n"/>
+      <c r="D62" s="32" t="n"/>
+      <c r="E62" s="32" t="n"/>
+      <c r="F62" s="32" t="n"/>
+    </row>
     <row r="63" ht="18" customHeight="1">
-      <c r="A63" s="34" t="inlineStr">
-        <is>
-          <t>Texto azul</t>
+      <c r="A63" s="36" t="inlineStr">
+        <is>
+          <t>Fondo gris claro</t>
         </is>
       </c>
       <c r="B63" s="35" t="inlineStr">
         <is>
-          <t>Celdas editables por el usuario (cantidad y precio unitario). El total se calcula automáticamente.</t>
+          <t>Subtotales y resumen del presupuesto.</t>
         </is>
       </c>
       <c r="C63" s="32" t="n"/>
@@ -1772,14 +1773,14 @@
       <c r="F63" s="32" t="n"/>
     </row>
     <row r="64" ht="18" customHeight="1">
-      <c r="A64" s="36" t="inlineStr">
-        <is>
-          <t>Fondo gris claro</t>
+      <c r="A64" s="37" t="inlineStr">
+        <is>
+          <t>Fondo gris oscuro</t>
         </is>
       </c>
       <c r="B64" s="35" t="inlineStr">
         <is>
-          <t>Subtotales y resumen del presupuesto.</t>
+          <t>Total general del presupuesto.</t>
         </is>
       </c>
       <c r="C64" s="32" t="n"/>
@@ -1787,79 +1788,62 @@
       <c r="E64" s="32" t="n"/>
       <c r="F64" s="32" t="n"/>
     </row>
-    <row r="65" ht="18" customHeight="1">
-      <c r="A65" s="37" t="inlineStr">
-        <is>
-          <t>Fondo gris oscuro</t>
-        </is>
-      </c>
-      <c r="B65" s="35" t="inlineStr">
-        <is>
-          <t>Total general del presupuesto.</t>
-        </is>
-      </c>
-      <c r="C65" s="32" t="n"/>
-      <c r="D65" s="32" t="n"/>
-      <c r="E65" s="32" t="n"/>
-      <c r="F65" s="32" t="n"/>
-    </row>
-    <row r="67" ht="34" customHeight="1"/>
-    <row r="68" ht="20" customHeight="1">
-      <c r="B68" s="38" t="inlineStr">
+    <row r="66" ht="34" customHeight="1"/>
+    <row r="67" ht="20" customHeight="1">
+      <c r="B67" s="38" t="inlineStr">
         <is>
           <t>Elaborado por</t>
         </is>
       </c>
-      <c r="C68" s="39" t="n"/>
-      <c r="E68" s="38" t="inlineStr">
+      <c r="C67" s="39" t="n"/>
+      <c r="E67" s="38" t="inlineStr">
         <is>
           <t>Aprobado por / Cliente</t>
         </is>
       </c>
-      <c r="F68" s="39" t="n"/>
+      <c r="F67" s="39" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="42">
+  <mergeCells count="41">
     <mergeCell ref="A54:F54"/>
     <mergeCell ref="A48:E48"/>
     <mergeCell ref="A24:E24"/>
     <mergeCell ref="C8:F8"/>
-    <mergeCell ref="E68:F68"/>
+    <mergeCell ref="B62:F62"/>
+    <mergeCell ref="E67:F67"/>
     <mergeCell ref="A49:E49"/>
     <mergeCell ref="C7:F7"/>
-    <mergeCell ref="A51:E51"/>
     <mergeCell ref="A45:E45"/>
     <mergeCell ref="A56:F56"/>
+    <mergeCell ref="F49"/>
     <mergeCell ref="A55:F55"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A57:F57"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A7:B7"/>
+    <mergeCell ref="B67:C67"/>
     <mergeCell ref="C6:F6"/>
     <mergeCell ref="A37:E37"/>
     <mergeCell ref="A46:E46"/>
-    <mergeCell ref="A62:F62"/>
     <mergeCell ref="C5:F5"/>
     <mergeCell ref="A53:F53"/>
     <mergeCell ref="A38:F38"/>
     <mergeCell ref="A50:E50"/>
     <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A52:F52"/>
     <mergeCell ref="C4:F4"/>
     <mergeCell ref="A44:F44"/>
     <mergeCell ref="A42:E42"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A47:E47"/>
     <mergeCell ref="A58:F58"/>
-    <mergeCell ref="F51"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A59:F59"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="B65:F65"/>
-    <mergeCell ref="B68:C68"/>
     <mergeCell ref="F50"/>
-    <mergeCell ref="A60:F60"/>
     <mergeCell ref="B64:F64"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A61:F61"/>
     <mergeCell ref="B63:F63"/>
     <mergeCell ref="A25:F25"/>
   </mergeCells>
@@ -2116,7 +2100,7 @@
       </c>
       <c r="C14" s="44" t="inlineStr">
         <is>
-          <t>Marco de tubo cuadrado de 1 1/2" chapa 14 con forro de lámina negra de 1/16" (4x8 pies). Uniones soldadas con electrodo 6011 de 3/32".</t>
+          <t>Marco de tubo cuadrado de 1 1/2" chapa 14 con forro de lámina negra de 1 mm (cal. 20, 4x8 pies). Uniones soldadas con electrodo 6011 de 3/32".</t>
         </is>
       </c>
       <c r="D14" s="44" t="inlineStr">

</xml_diff>

<commit_message>
Rediseñar leyenda de colores del presupuesto para que sea legible
La etiqueta iba en la columna A (angosta, ancho 7) y el texto se cortaba.
Ahora la col A es solo un cuadrito de muestra del color y la etiqueta +
descripcion van en columnas anchas, sin texto cortado.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018cUG4L4bYGYeGqZHWF8NkF
</commit_message>
<xml_diff>
--- a/Presupuesto_Muro_Perimetral.xlsx
+++ b/Presupuesto_Muro_Perimetral.xlsx
@@ -198,7 +198,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -286,16 +286,19 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1752,68 +1755,72 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="18" customHeight="1">
+    <row r="63" ht="36" customHeight="1">
       <c r="A63" s="34" t="inlineStr">
         <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="B63" s="35" t="inlineStr">
+        <is>
           <t>Texto azul</t>
         </is>
       </c>
-      <c r="B63" s="35" t="inlineStr">
-        <is>
-          <t>Celdas editables por el usuario (cantidad y precio unitario). El total se calcula automáticamente.</t>
-        </is>
-      </c>
-      <c r="C63" s="32" t="n"/>
+      <c r="C63" s="36" t="inlineStr">
+        <is>
+          <t>Celdas que puede editar (cantidad y precio unitario); el total se calcula solo.</t>
+        </is>
+      </c>
       <c r="D63" s="32" t="n"/>
       <c r="E63" s="32" t="n"/>
       <c r="F63" s="32" t="n"/>
     </row>
-    <row r="64" ht="18" customHeight="1">
-      <c r="A64" s="36" t="inlineStr">
+    <row r="64" ht="21" customHeight="1">
+      <c r="A64" s="37" t="inlineStr"/>
+      <c r="B64" s="35" t="inlineStr">
         <is>
           <t>Fondo gris claro</t>
         </is>
       </c>
-      <c r="B64" s="35" t="inlineStr">
+      <c r="C64" s="36" t="inlineStr">
         <is>
           <t>Subtotales y resumen del presupuesto.</t>
         </is>
       </c>
-      <c r="C64" s="32" t="n"/>
       <c r="D64" s="32" t="n"/>
       <c r="E64" s="32" t="n"/>
       <c r="F64" s="32" t="n"/>
     </row>
-    <row r="65" ht="18" customHeight="1">
-      <c r="A65" s="37" t="inlineStr">
+    <row r="65" ht="21" customHeight="1">
+      <c r="A65" s="38" t="inlineStr"/>
+      <c r="B65" s="35" t="inlineStr">
         <is>
           <t>Fondo gris oscuro</t>
         </is>
       </c>
-      <c r="B65" s="35" t="inlineStr">
+      <c r="C65" s="36" t="inlineStr">
         <is>
           <t>Total general del presupuesto.</t>
         </is>
       </c>
-      <c r="C65" s="32" t="n"/>
       <c r="D65" s="32" t="n"/>
       <c r="E65" s="32" t="n"/>
       <c r="F65" s="32" t="n"/>
     </row>
     <row r="67" ht="34" customHeight="1"/>
     <row r="68" ht="20" customHeight="1">
-      <c r="B68" s="38" t="inlineStr">
+      <c r="B68" s="39" t="inlineStr">
         <is>
           <t>Elaborado por</t>
         </is>
       </c>
-      <c r="C68" s="39" t="n"/>
-      <c r="E68" s="38" t="inlineStr">
+      <c r="C68" s="40" t="n"/>
+      <c r="E68" s="39" t="inlineStr">
         <is>
           <t>Aprobado por / Cliente</t>
         </is>
       </c>
-      <c r="F68" s="39" t="n"/>
+      <c r="F68" s="40" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="42">
@@ -1842,22 +1849,22 @@
     <mergeCell ref="A50:E50"/>
     <mergeCell ref="A10:F10"/>
     <mergeCell ref="A52:F52"/>
+    <mergeCell ref="C64:F64"/>
     <mergeCell ref="C4:F4"/>
     <mergeCell ref="A44:F44"/>
     <mergeCell ref="A42:E42"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A47:E47"/>
     <mergeCell ref="A58:F58"/>
+    <mergeCell ref="C63:F63"/>
+    <mergeCell ref="C65:F65"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A59:F59"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="B65:F65"/>
     <mergeCell ref="B68:C68"/>
     <mergeCell ref="F50"/>
     <mergeCell ref="A60:F60"/>
-    <mergeCell ref="B64:F64"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B63:F63"/>
     <mergeCell ref="A25:F25"/>
   </mergeCells>
   <dataValidations count="1">
@@ -1923,10 +1930,10 @@
       </c>
     </row>
     <row r="5" ht="68" customHeight="1">
-      <c r="A5" s="40" t="n">
+      <c r="A5" s="41" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="41" t="inlineStr">
+      <c r="B5" s="42" t="inlineStr">
         <is>
           <t>Muro existente (base)</t>
         </is>
@@ -1943,30 +1950,30 @@
       </c>
     </row>
     <row r="6" ht="53" customHeight="1">
-      <c r="A6" s="42" t="n">
+      <c r="A6" s="43" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="43" t="inlineStr">
+      <c r="B6" s="44" t="inlineStr">
         <is>
           <t>Unidad de mampostería</t>
         </is>
       </c>
-      <c r="C6" s="44" t="inlineStr">
+      <c r="C6" s="45" t="inlineStr">
         <is>
           <t>Bloque de concreto hueco de 6" (nominal 15x20x40 cm), asentado a soga con junta de 1.0 a 1.5 cm. Resistencia mínima recomendada f'm según uso estructural.</t>
         </is>
       </c>
-      <c r="D6" s="44" t="inlineStr">
+      <c r="D6" s="45" t="inlineStr">
         <is>
           <t>ASTM C90 / NTON 12 008-09</t>
         </is>
       </c>
     </row>
     <row r="7" ht="53" customHeight="1">
-      <c r="A7" s="40" t="n">
+      <c r="A7" s="41" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="41" t="inlineStr">
+      <c r="B7" s="42" t="inlineStr">
         <is>
           <t>Mortero de pega</t>
         </is>
@@ -1983,30 +1990,30 @@
       </c>
     </row>
     <row r="8" ht="53" customHeight="1">
-      <c r="A8" s="42" t="n">
+      <c r="A8" s="43" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="43" t="inlineStr">
+      <c r="B8" s="44" t="inlineStr">
         <is>
           <t>Concreto de relleno / columnas</t>
         </is>
       </c>
-      <c r="C8" s="44" t="inlineStr">
+      <c r="C8" s="45" t="inlineStr">
         <is>
           <t>Concreto en celdas reforzadas y columnas de confinamiento, proporción 1:2:2 (cemento:arena:piedrín de 1/2"), resistencia f'c ≥ 3000 psi (210 kg/cm²). Vibrado o chuzeado.</t>
         </is>
       </c>
-      <c r="D8" s="44" t="inlineStr">
+      <c r="D8" s="45" t="inlineStr">
         <is>
           <t>ACI 318 / RNC-07</t>
         </is>
       </c>
     </row>
     <row r="9" ht="53" customHeight="1">
-      <c r="A9" s="40" t="n">
+      <c r="A9" s="41" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="41" t="inlineStr">
+      <c r="B9" s="42" t="inlineStr">
         <is>
           <t>Refuerzo vertical</t>
         </is>
@@ -2023,30 +2030,30 @@
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
-      <c r="A10" s="42" t="n">
+      <c r="A10" s="43" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="43" t="inlineStr">
+      <c r="B10" s="44" t="inlineStr">
         <is>
           <t>Refuerzo transversal</t>
         </is>
       </c>
-      <c r="C10" s="44" t="inlineStr">
+      <c r="C10" s="45" t="inlineStr">
         <is>
           <t>Estribos de 1/4" de 10x10 cm, separación típica cada 15-20 cm en columnas y confinamiento de viga. Ganchos a 135°.</t>
         </is>
       </c>
-      <c r="D10" s="44" t="inlineStr">
+      <c r="D10" s="45" t="inlineStr">
         <is>
           <t>ACI 318 / RNC-07</t>
         </is>
       </c>
     </row>
     <row r="11" ht="53" customHeight="1">
-      <c r="A11" s="40" t="n">
+      <c r="A11" s="41" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="41" t="inlineStr">
+      <c r="B11" s="42" t="inlineStr">
         <is>
           <t>Viga corona / solera</t>
         </is>
@@ -2063,30 +2070,30 @@
       </c>
     </row>
     <row r="12" ht="53" customHeight="1">
-      <c r="A12" s="42" t="n">
+      <c r="A12" s="43" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="43" t="inlineStr">
+      <c r="B12" s="44" t="inlineStr">
         <is>
           <t>Amarres y fijación</t>
         </is>
       </c>
-      <c r="C12" s="44" t="inlineStr">
+      <c r="C12" s="45" t="inlineStr">
         <is>
           <t>Alambre de amarre recocido cal. 18 para el armado del acero. Clavos corrientes y de acero de 2 1/2" para la formaleta de madera (tabla y regla de pino).</t>
         </is>
       </c>
-      <c r="D12" s="44" t="inlineStr">
+      <c r="D12" s="45" t="inlineStr">
         <is>
           <t>Práctica constructiva</t>
         </is>
       </c>
     </row>
     <row r="13" ht="53" customHeight="1">
-      <c r="A13" s="40" t="n">
+      <c r="A13" s="41" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="41" t="inlineStr">
+      <c r="B13" s="42" t="inlineStr">
         <is>
           <t>Encofrado / formaleta</t>
         </is>
@@ -2103,30 +2110,30 @@
       </c>
     </row>
     <row r="14" ht="38" customHeight="1">
-      <c r="A14" s="42" t="n">
+      <c r="A14" s="43" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="43" t="inlineStr">
+      <c r="B14" s="44" t="inlineStr">
         <is>
           <t>Estructura del portón</t>
         </is>
       </c>
-      <c r="C14" s="44" t="inlineStr">
+      <c r="C14" s="45" t="inlineStr">
         <is>
           <t>Marco de tubo cuadrado de 1 1/2" chapa 14 con forro de lámina negra de 1 mm (cal. 20, 4x8 pies). Uniones soldadas con electrodo 6011 de 3/32".</t>
         </is>
       </c>
-      <c r="D14" s="44" t="inlineStr">
+      <c r="D14" s="45" t="inlineStr">
         <is>
           <t>AWS D1.1 / práctica de taller</t>
         </is>
       </c>
     </row>
     <row r="15" ht="38" customHeight="1">
-      <c r="A15" s="40" t="n">
+      <c r="A15" s="41" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="41" t="inlineStr">
+      <c r="B15" s="42" t="inlineStr">
         <is>
           <t>Herrajes del portón</t>
         </is>
@@ -2143,30 +2150,30 @@
       </c>
     </row>
     <row r="16" ht="38" customHeight="1">
-      <c r="A16" s="42" t="n">
+      <c r="A16" s="43" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="43" t="inlineStr">
+      <c r="B16" s="44" t="inlineStr">
         <is>
           <t>Protección anticorrosiva</t>
         </is>
       </c>
-      <c r="C16" s="44" t="inlineStr">
+      <c r="C16" s="45" t="inlineStr">
         <is>
           <t>Limpieza de escoria y desengrase; una mano de pintura anticorrosiva (base) diluida con thinner sobre el portón y los elementos metálicos.</t>
         </is>
       </c>
-      <c r="D16" s="44" t="inlineStr">
+      <c r="D16" s="45" t="inlineStr">
         <is>
           <t>SSPC-SP2 / ficha técnica</t>
         </is>
       </c>
     </row>
     <row r="17" ht="38" customHeight="1">
-      <c r="A17" s="40" t="n">
+      <c r="A17" s="41" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="41" t="inlineStr">
+      <c r="B17" s="42" t="inlineStr">
         <is>
           <t>Concertina / serpentina</t>
         </is>
@@ -2183,30 +2190,30 @@
       </c>
     </row>
     <row r="18" ht="38" customHeight="1">
-      <c r="A18" s="42" t="n">
+      <c r="A18" s="43" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="43" t="inlineStr">
+      <c r="B18" s="44" t="inlineStr">
         <is>
           <t>Corte de metal</t>
         </is>
       </c>
-      <c r="C18" s="44" t="inlineStr">
+      <c r="C18" s="45" t="inlineStr">
         <is>
           <t>Corte de tubo y lámina con disco de corte fino de 7" para acero, con equipo y equipo de protección personal adecuado.</t>
         </is>
       </c>
-      <c r="D18" s="44" t="inlineStr">
+      <c r="D18" s="45" t="inlineStr">
         <is>
           <t>Seguridad ocupacional</t>
         </is>
       </c>
     </row>
     <row r="19" ht="53" customHeight="1">
-      <c r="A19" s="40" t="n">
+      <c r="A19" s="41" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="41" t="inlineStr">
+      <c r="B19" s="42" t="inlineStr">
         <is>
           <t>Curado</t>
         </is>
@@ -2223,7 +2230,7 @@
       </c>
     </row>
     <row r="21" ht="46" customHeight="1">
-      <c r="A21" s="45" t="inlineStr">
+      <c r="A21" s="46" t="inlineStr">
         <is>
           <t>Nota: Este cuadro es de carácter referencial y de buena práctica constructiva. Las secciones, separaciones de refuerzo y resistencias definitivas deben ser validadas por el ingeniero responsable según el Reglamento Nacional de la Construcción (RNC-07) de Nicaragua.</t>
         </is>

</xml_diff>

<commit_message>
Eliminar leyenda de colores del presupuesto para ahorrar espacio
Las firmas pasan a ubicarse justo despues de las observaciones.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018cUG4L4bYGYeGqZHWF8NkF
</commit_message>
<xml_diff>
--- a/Presupuesto_Muro_Perimetral.xlsx
+++ b/Presupuesto_Muro_Perimetral.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Presupuesto'!$11:$11</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Presupuesto'!$A$1:$F$68</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Presupuesto'!$A$1:$F$63</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Especificaciones Técnicas'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Especificaciones Técnicas'!$A$1:$D$21</definedName>
   </definedNames>
@@ -29,7 +29,7 @@
     <numFmt numFmtId="167" formatCode="&quot;C$&quot;#,##0.00"/>
     <numFmt numFmtId="168" formatCode="&quot;US$ &quot;#,##0.00"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -97,29 +97,11 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001F4E79"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="000000FF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -161,11 +143,6 @@
         <fgColor rgb="00595959"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -198,7 +175,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -282,24 +259,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -307,13 +266,13 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -687,7 +646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1748,87 +1707,27 @@
       <c r="E60" s="32" t="n"/>
       <c r="F60" s="32" t="n"/>
     </row>
-    <row r="62" ht="20" customHeight="1">
-      <c r="A62" s="33" t="inlineStr">
-        <is>
-          <t>LEYENDA DE COLORES</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="36" customHeight="1">
-      <c r="A63" s="34" t="inlineStr">
-        <is>
-          <t>123</t>
-        </is>
-      </c>
-      <c r="B63" s="35" t="inlineStr">
-        <is>
-          <t>Texto azul</t>
-        </is>
-      </c>
-      <c r="C63" s="36" t="inlineStr">
-        <is>
-          <t>Celdas que puede editar (cantidad y precio unitario); el total se calcula solo.</t>
-        </is>
-      </c>
-      <c r="D63" s="32" t="n"/>
-      <c r="E63" s="32" t="n"/>
-      <c r="F63" s="32" t="n"/>
-    </row>
-    <row r="64" ht="21" customHeight="1">
-      <c r="A64" s="37" t="inlineStr"/>
-      <c r="B64" s="35" t="inlineStr">
-        <is>
-          <t>Fondo gris claro</t>
-        </is>
-      </c>
-      <c r="C64" s="36" t="inlineStr">
-        <is>
-          <t>Subtotales y resumen del presupuesto.</t>
-        </is>
-      </c>
-      <c r="D64" s="32" t="n"/>
-      <c r="E64" s="32" t="n"/>
-      <c r="F64" s="32" t="n"/>
-    </row>
-    <row r="65" ht="21" customHeight="1">
-      <c r="A65" s="38" t="inlineStr"/>
-      <c r="B65" s="35" t="inlineStr">
-        <is>
-          <t>Fondo gris oscuro</t>
-        </is>
-      </c>
-      <c r="C65" s="36" t="inlineStr">
-        <is>
-          <t>Total general del presupuesto.</t>
-        </is>
-      </c>
-      <c r="D65" s="32" t="n"/>
-      <c r="E65" s="32" t="n"/>
-      <c r="F65" s="32" t="n"/>
-    </row>
-    <row r="67" ht="34" customHeight="1"/>
-    <row r="68" ht="20" customHeight="1">
-      <c r="B68" s="39" t="inlineStr">
+    <row r="62" ht="34" customHeight="1"/>
+    <row r="63" ht="20" customHeight="1">
+      <c r="B63" s="33" t="inlineStr">
         <is>
           <t>Elaborado por</t>
         </is>
       </c>
-      <c r="C68" s="40" t="n"/>
-      <c r="E68" s="39" t="inlineStr">
+      <c r="C63" s="34" t="n"/>
+      <c r="E63" s="33" t="inlineStr">
         <is>
           <t>Aprobado por / Cliente</t>
         </is>
       </c>
-      <c r="F68" s="40" t="n"/>
+      <c r="F63" s="34" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="42">
+  <mergeCells count="38">
     <mergeCell ref="A54:F54"/>
     <mergeCell ref="A48:E48"/>
     <mergeCell ref="A24:E24"/>
     <mergeCell ref="C8:F8"/>
-    <mergeCell ref="E68:F68"/>
     <mergeCell ref="A49:E49"/>
     <mergeCell ref="C7:F7"/>
     <mergeCell ref="A45:E45"/>
@@ -1839,32 +1738,29 @@
     <mergeCell ref="A57:F57"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A7:B7"/>
+    <mergeCell ref="E63:F63"/>
     <mergeCell ref="C6:F6"/>
     <mergeCell ref="A37:E37"/>
     <mergeCell ref="A46:E46"/>
-    <mergeCell ref="A62:F62"/>
     <mergeCell ref="C5:F5"/>
     <mergeCell ref="A53:F53"/>
     <mergeCell ref="A38:F38"/>
     <mergeCell ref="A50:E50"/>
     <mergeCell ref="A10:F10"/>
     <mergeCell ref="A52:F52"/>
-    <mergeCell ref="C64:F64"/>
     <mergeCell ref="C4:F4"/>
     <mergeCell ref="A44:F44"/>
     <mergeCell ref="A42:E42"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A47:E47"/>
     <mergeCell ref="A58:F58"/>
-    <mergeCell ref="C63:F63"/>
-    <mergeCell ref="C65:F65"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A59:F59"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="B68:C68"/>
     <mergeCell ref="F50"/>
     <mergeCell ref="A60:F60"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B63:C63"/>
     <mergeCell ref="A25:F25"/>
   </mergeCells>
   <dataValidations count="1">
@@ -1930,10 +1826,10 @@
       </c>
     </row>
     <row r="5" ht="68" customHeight="1">
-      <c r="A5" s="41" t="n">
+      <c r="A5" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="42" t="inlineStr">
+      <c r="B5" s="36" t="inlineStr">
         <is>
           <t>Muro existente (base)</t>
         </is>
@@ -1950,30 +1846,30 @@
       </c>
     </row>
     <row r="6" ht="53" customHeight="1">
-      <c r="A6" s="43" t="n">
+      <c r="A6" s="37" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="44" t="inlineStr">
+      <c r="B6" s="38" t="inlineStr">
         <is>
           <t>Unidad de mampostería</t>
         </is>
       </c>
-      <c r="C6" s="45" t="inlineStr">
+      <c r="C6" s="39" t="inlineStr">
         <is>
           <t>Bloque de concreto hueco de 6" (nominal 15x20x40 cm), asentado a soga con junta de 1.0 a 1.5 cm. Resistencia mínima recomendada f'm según uso estructural.</t>
         </is>
       </c>
-      <c r="D6" s="45" t="inlineStr">
+      <c r="D6" s="39" t="inlineStr">
         <is>
           <t>ASTM C90 / NTON 12 008-09</t>
         </is>
       </c>
     </row>
     <row r="7" ht="53" customHeight="1">
-      <c r="A7" s="41" t="n">
+      <c r="A7" s="35" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="42" t="inlineStr">
+      <c r="B7" s="36" t="inlineStr">
         <is>
           <t>Mortero de pega</t>
         </is>
@@ -1990,30 +1886,30 @@
       </c>
     </row>
     <row r="8" ht="53" customHeight="1">
-      <c r="A8" s="43" t="n">
+      <c r="A8" s="37" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="44" t="inlineStr">
+      <c r="B8" s="38" t="inlineStr">
         <is>
           <t>Concreto de relleno / columnas</t>
         </is>
       </c>
-      <c r="C8" s="45" t="inlineStr">
+      <c r="C8" s="39" t="inlineStr">
         <is>
           <t>Concreto en celdas reforzadas y columnas de confinamiento, proporción 1:2:2 (cemento:arena:piedrín de 1/2"), resistencia f'c ≥ 3000 psi (210 kg/cm²). Vibrado o chuzeado.</t>
         </is>
       </c>
-      <c r="D8" s="45" t="inlineStr">
+      <c r="D8" s="39" t="inlineStr">
         <is>
           <t>ACI 318 / RNC-07</t>
         </is>
       </c>
     </row>
     <row r="9" ht="53" customHeight="1">
-      <c r="A9" s="41" t="n">
+      <c r="A9" s="35" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="42" t="inlineStr">
+      <c r="B9" s="36" t="inlineStr">
         <is>
           <t>Refuerzo vertical</t>
         </is>
@@ -2030,30 +1926,30 @@
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
-      <c r="A10" s="43" t="n">
+      <c r="A10" s="37" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="44" t="inlineStr">
+      <c r="B10" s="38" t="inlineStr">
         <is>
           <t>Refuerzo transversal</t>
         </is>
       </c>
-      <c r="C10" s="45" t="inlineStr">
+      <c r="C10" s="39" t="inlineStr">
         <is>
           <t>Estribos de 1/4" de 10x10 cm, separación típica cada 15-20 cm en columnas y confinamiento de viga. Ganchos a 135°.</t>
         </is>
       </c>
-      <c r="D10" s="45" t="inlineStr">
+      <c r="D10" s="39" t="inlineStr">
         <is>
           <t>ACI 318 / RNC-07</t>
         </is>
       </c>
     </row>
     <row r="11" ht="53" customHeight="1">
-      <c r="A11" s="41" t="n">
+      <c r="A11" s="35" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="42" t="inlineStr">
+      <c r="B11" s="36" t="inlineStr">
         <is>
           <t>Viga corona / solera</t>
         </is>
@@ -2070,30 +1966,30 @@
       </c>
     </row>
     <row r="12" ht="53" customHeight="1">
-      <c r="A12" s="43" t="n">
+      <c r="A12" s="37" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="44" t="inlineStr">
+      <c r="B12" s="38" t="inlineStr">
         <is>
           <t>Amarres y fijación</t>
         </is>
       </c>
-      <c r="C12" s="45" t="inlineStr">
+      <c r="C12" s="39" t="inlineStr">
         <is>
           <t>Alambre de amarre recocido cal. 18 para el armado del acero. Clavos corrientes y de acero de 2 1/2" para la formaleta de madera (tabla y regla de pino).</t>
         </is>
       </c>
-      <c r="D12" s="45" t="inlineStr">
+      <c r="D12" s="39" t="inlineStr">
         <is>
           <t>Práctica constructiva</t>
         </is>
       </c>
     </row>
     <row r="13" ht="53" customHeight="1">
-      <c r="A13" s="41" t="n">
+      <c r="A13" s="35" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="42" t="inlineStr">
+      <c r="B13" s="36" t="inlineStr">
         <is>
           <t>Encofrado / formaleta</t>
         </is>
@@ -2110,30 +2006,30 @@
       </c>
     </row>
     <row r="14" ht="38" customHeight="1">
-      <c r="A14" s="43" t="n">
+      <c r="A14" s="37" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="44" t="inlineStr">
+      <c r="B14" s="38" t="inlineStr">
         <is>
           <t>Estructura del portón</t>
         </is>
       </c>
-      <c r="C14" s="45" t="inlineStr">
+      <c r="C14" s="39" t="inlineStr">
         <is>
           <t>Marco de tubo cuadrado de 1 1/2" chapa 14 con forro de lámina negra de 1 mm (cal. 20, 4x8 pies). Uniones soldadas con electrodo 6011 de 3/32".</t>
         </is>
       </c>
-      <c r="D14" s="45" t="inlineStr">
+      <c r="D14" s="39" t="inlineStr">
         <is>
           <t>AWS D1.1 / práctica de taller</t>
         </is>
       </c>
     </row>
     <row r="15" ht="38" customHeight="1">
-      <c r="A15" s="41" t="n">
+      <c r="A15" s="35" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="42" t="inlineStr">
+      <c r="B15" s="36" t="inlineStr">
         <is>
           <t>Herrajes del portón</t>
         </is>
@@ -2150,30 +2046,30 @@
       </c>
     </row>
     <row r="16" ht="38" customHeight="1">
-      <c r="A16" s="43" t="n">
+      <c r="A16" s="37" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="44" t="inlineStr">
+      <c r="B16" s="38" t="inlineStr">
         <is>
           <t>Protección anticorrosiva</t>
         </is>
       </c>
-      <c r="C16" s="45" t="inlineStr">
+      <c r="C16" s="39" t="inlineStr">
         <is>
           <t>Limpieza de escoria y desengrase; una mano de pintura anticorrosiva (base) diluida con thinner sobre el portón y los elementos metálicos.</t>
         </is>
       </c>
-      <c r="D16" s="45" t="inlineStr">
+      <c r="D16" s="39" t="inlineStr">
         <is>
           <t>SSPC-SP2 / ficha técnica</t>
         </is>
       </c>
     </row>
     <row r="17" ht="38" customHeight="1">
-      <c r="A17" s="41" t="n">
+      <c r="A17" s="35" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="42" t="inlineStr">
+      <c r="B17" s="36" t="inlineStr">
         <is>
           <t>Concertina / serpentina</t>
         </is>
@@ -2190,30 +2086,30 @@
       </c>
     </row>
     <row r="18" ht="38" customHeight="1">
-      <c r="A18" s="43" t="n">
+      <c r="A18" s="37" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="44" t="inlineStr">
+      <c r="B18" s="38" t="inlineStr">
         <is>
           <t>Corte de metal</t>
         </is>
       </c>
-      <c r="C18" s="45" t="inlineStr">
+      <c r="C18" s="39" t="inlineStr">
         <is>
           <t>Corte de tubo y lámina con disco de corte fino de 7" para acero, con equipo y equipo de protección personal adecuado.</t>
         </is>
       </c>
-      <c r="D18" s="45" t="inlineStr">
+      <c r="D18" s="39" t="inlineStr">
         <is>
           <t>Seguridad ocupacional</t>
         </is>
       </c>
     </row>
     <row r="19" ht="53" customHeight="1">
-      <c r="A19" s="41" t="n">
+      <c r="A19" s="35" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="42" t="inlineStr">
+      <c r="B19" s="36" t="inlineStr">
         <is>
           <t>Curado</t>
         </is>
@@ -2230,7 +2126,7 @@
       </c>
     </row>
     <row r="21" ht="46" customHeight="1">
-      <c r="A21" s="46" t="inlineStr">
+      <c r="A21" s="40" t="inlineStr">
         <is>
           <t>Nota: Este cuadro es de carácter referencial y de buena práctica constructiva. Las secciones, separaciones de refuerzo y resistencias definitivas deben ser validadas por el ingeniero responsable según el Reglamento Nacional de la Construcción (RNC-07) de Nicaragua.</t>
         </is>

</xml_diff>